<commit_message>
The old null model analyses based on a regional pool with the 13 seasonal bee species (that might not be active during our sampling time) removed were moved to scratch and rerun with the cleaned up 2025 dataset.
</commit_message>
<xml_diff>
--- a/Analysiswithoutseasonalbeestest/btraits_23.xlsx
+++ b/Analysiswithoutseasonalbeestest/btraits_23.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ohio_Bees\Analysiswithoutseasonalbeestest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7371B5F7-DF53-4E0B-A007-3F36C38ABD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78BD5DC5-D413-49CA-ACD8-37B106BAEE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{89B5C4F4-CBB4-4BE3-96F6-CA7CA2C4E704}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="353">
   <si>
     <t>BodyLength</t>
   </si>
@@ -1031,9 +1031,6 @@
   </si>
   <si>
     <t>Sphecodeslevis</t>
-  </si>
-  <si>
-    <t>Sphecodesmandibularis</t>
   </si>
   <si>
     <t>Sphecodesminor</t>
@@ -1942,7 +1939,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66E3C8A-BF41-4212-AFF6-1256B7C85012}">
-  <dimension ref="A1:F350"/>
+  <dimension ref="A1:F349"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
@@ -8592,7 +8589,7 @@
         <v>337</v>
       </c>
       <c r="B334">
-        <v>6.95</v>
+        <v>6.8</v>
       </c>
       <c r="C334">
         <v>0</v>
@@ -8612,7 +8609,7 @@
         <v>338</v>
       </c>
       <c r="B335">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="C335">
         <v>0</v>
@@ -8632,7 +8629,7 @@
         <v>339</v>
       </c>
       <c r="B336">
-        <v>7</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="C336">
         <v>0</v>
@@ -8652,7 +8649,7 @@
         <v>340</v>
       </c>
       <c r="B337">
-        <v>9.1999999999999993</v>
+        <v>7.5</v>
       </c>
       <c r="C337">
         <v>0</v>
@@ -8672,13 +8669,13 @@
         <v>341</v>
       </c>
       <c r="B338">
-        <v>7.5</v>
+        <v>6.7</v>
       </c>
       <c r="C338">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D338">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E338">
         <v>4</v>
@@ -8692,7 +8689,7 @@
         <v>342</v>
       </c>
       <c r="B339">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="C339">
         <v>1</v>
@@ -8712,7 +8709,7 @@
         <v>343</v>
       </c>
       <c r="B340">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C340">
         <v>1</v>
@@ -8732,7 +8729,7 @@
         <v>344</v>
       </c>
       <c r="B341">
-        <v>8</v>
+        <v>9.6300000000000008</v>
       </c>
       <c r="C341">
         <v>1</v>
@@ -8752,16 +8749,16 @@
         <v>345</v>
       </c>
       <c r="B342">
-        <v>9.6300000000000008</v>
+        <v>15.25</v>
       </c>
       <c r="C342">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D342">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E342">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F342">
         <v>0</v>
@@ -8772,16 +8769,16 @@
         <v>346</v>
       </c>
       <c r="B343">
-        <v>15.25</v>
+        <v>11.5</v>
       </c>
       <c r="C343">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D343">
         <v>1</v>
       </c>
       <c r="E343">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F343">
         <v>0</v>
@@ -8792,7 +8789,7 @@
         <v>347</v>
       </c>
       <c r="B344">
-        <v>11.5</v>
+        <v>11</v>
       </c>
       <c r="C344">
         <v>0</v>
@@ -8812,7 +8809,7 @@
         <v>348</v>
       </c>
       <c r="B345">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C345">
         <v>0</v>
@@ -8832,7 +8829,7 @@
         <v>349</v>
       </c>
       <c r="B346">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C346">
         <v>0</v>
@@ -8852,7 +8849,7 @@
         <v>350</v>
       </c>
       <c r="B347">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C347">
         <v>0</v>
@@ -8872,16 +8869,16 @@
         <v>351</v>
       </c>
       <c r="B348">
-        <v>12</v>
+        <v>15.38</v>
       </c>
       <c r="C348">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D348">
         <v>1</v>
       </c>
       <c r="E348">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F348">
         <v>0</v>
@@ -8892,38 +8889,18 @@
         <v>352</v>
       </c>
       <c r="B349">
-        <v>15.38</v>
+        <v>20</v>
       </c>
       <c r="C349">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D349">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E349">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F349">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="350" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A350" t="s">
-        <v>353</v>
-      </c>
-      <c r="B350">
-        <v>20</v>
-      </c>
-      <c r="C350">
-        <v>1</v>
-      </c>
-      <c r="D350">
-        <v>5</v>
-      </c>
-      <c r="E350">
-        <v>1</v>
-      </c>
-      <c r="F350">
         <v>0</v>
       </c>
     </row>

</xml_diff>